<commit_message>
Three-agent review of Module 1 (content, aesthetics, embeds and videos); include latest descriptives save
Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01TNVxQFJXojPDm4Z5hNnmdq
</commit_message>
<xml_diff>
--- a/textbook_examples/mod01_descriptives.xlsx
+++ b/textbook_examples/mod01_descriptives.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://usaskca1-my.sharepoint.com/personal/pjs998_usask_ca/Documents/Teaching/261/2026/textbook_261/textbook_examples/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="157" documentId="8_{40A48D82-9896-1D40-A33B-1B9FE8A350F6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{732E23D8-6945-2748-A8FD-228D7BB3B759}"/>
+  <xr:revisionPtr revIDLastSave="159" documentId="8_{40A48D82-9896-1D40-A33B-1B9FE8A350F6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{FB1EDDDA-D220-7F48-80FF-7FEA6C4C0826}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="0" windowWidth="38400" windowHeight="21600" activeTab="9" xr2:uid="{E0A39ED0-7C98-1C4C-834F-3D01DA12686E}"/>
   </bookViews>
@@ -1469,162 +1469,6 @@
 </cx:chartSpace>
 </file>
 
-<file path=xl/charts/chartEx4.xml><?xml version="1.0" encoding="utf-8"?>
-<cx:chartSpace xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:cx="http://schemas.microsoft.com/office/drawing/2014/chartex">
-  <cx:chartData>
-    <cx:data id="0">
-      <cx:numDim type="val">
-        <cx:f>_xlchart.v1.4</cx:f>
-      </cx:numDim>
-    </cx:data>
-  </cx:chartData>
-  <cx:chart>
-    <cx:title pos="t" align="ctr" overlay="0">
-      <cx:tx>
-        <cx:txData>
-          <cx:v>Histogram of barley variety yields</cx:v>
-        </cx:txData>
-      </cx:tx>
-      <cx:txPr>
-        <a:bodyPr spcFirstLastPara="1" vertOverflow="ellipsis" horzOverflow="overflow" wrap="square" lIns="0" tIns="0" rIns="0" bIns="0" anchor="ctr" anchorCtr="1"/>
-        <a:lstStyle/>
-        <a:p>
-          <a:pPr algn="ctr" rtl="0">
-            <a:defRPr/>
-          </a:pPr>
-          <a:r>
-            <a:rPr lang="en-US" sz="1400" b="0" i="0" u="none" strike="noStrike" baseline="0">
-              <a:solidFill>
-                <a:sysClr val="windowText" lastClr="000000">
-                  <a:lumMod val="65000"/>
-                  <a:lumOff val="35000"/>
-                </a:sysClr>
-              </a:solidFill>
-              <a:latin typeface="Aptos Narrow" panose="02110004020202020204"/>
-            </a:rPr>
-            <a:t>Histogram of barley variety yields</a:t>
-          </a:r>
-        </a:p>
-      </cx:txPr>
-    </cx:title>
-    <cx:plotArea>
-      <cx:plotAreaRegion>
-        <cx:series layoutId="clusteredColumn" uniqueId="{00000000-0FC2-0947-9B1F-769ECEC59389}">
-          <cx:dataPt idx="1"/>
-          <cx:dataId val="0"/>
-          <cx:layoutPr>
-            <cx:binning intervalClosed="r" underflow="55" overflow="100">
-              <cx:binCount val="5"/>
-            </cx:binning>
-          </cx:layoutPr>
-        </cx:series>
-      </cx:plotAreaRegion>
-      <cx:axis id="0">
-        <cx:catScaling gapWidth="0"/>
-        <cx:title>
-          <cx:tx>
-            <cx:txData>
-              <cx:v>Yields (bu/acres)</cx:v>
-            </cx:txData>
-          </cx:tx>
-          <cx:txPr>
-            <a:bodyPr spcFirstLastPara="1" vertOverflow="ellipsis" horzOverflow="overflow" wrap="square" lIns="0" tIns="0" rIns="0" bIns="0" anchor="ctr" anchorCtr="1"/>
-            <a:lstStyle/>
-            <a:p>
-              <a:pPr algn="ctr" rtl="0">
-                <a:defRPr sz="1400"/>
-              </a:pPr>
-              <a:r>
-                <a:rPr lang="en-US" sz="1400" b="0" i="0" u="none" strike="noStrike" baseline="0">
-                  <a:solidFill>
-                    <a:sysClr val="windowText" lastClr="000000">
-                      <a:lumMod val="65000"/>
-                      <a:lumOff val="35000"/>
-                    </a:sysClr>
-                  </a:solidFill>
-                  <a:latin typeface="Aptos Narrow" panose="02110004020202020204"/>
-                </a:rPr>
-                <a:t>Yields (bu/acres)</a:t>
-              </a:r>
-            </a:p>
-          </cx:txPr>
-        </cx:title>
-        <cx:tickLabels/>
-        <cx:txPr>
-          <a:bodyPr spcFirstLastPara="1" vertOverflow="ellipsis" horzOverflow="overflow" wrap="square" lIns="0" tIns="0" rIns="0" bIns="0" anchor="ctr" anchorCtr="1"/>
-          <a:lstStyle/>
-          <a:p>
-            <a:pPr algn="ctr" rtl="0">
-              <a:defRPr sz="1100"/>
-            </a:pPr>
-            <a:endParaRPr lang="en-US" sz="1100" b="0" i="0" u="none" strike="noStrike" baseline="0">
-              <a:solidFill>
-                <a:sysClr val="windowText" lastClr="000000">
-                  <a:lumMod val="65000"/>
-                  <a:lumOff val="35000"/>
-                </a:sysClr>
-              </a:solidFill>
-              <a:latin typeface="Aptos Narrow" panose="02110004020202020204"/>
-            </a:endParaRPr>
-          </a:p>
-        </cx:txPr>
-      </cx:axis>
-      <cx:axis id="1">
-        <cx:valScaling/>
-        <cx:title>
-          <cx:tx>
-            <cx:txData>
-              <cx:v>Number of varieties</cx:v>
-            </cx:txData>
-          </cx:tx>
-          <cx:txPr>
-            <a:bodyPr spcFirstLastPara="1" vertOverflow="ellipsis" horzOverflow="overflow" wrap="square" lIns="0" tIns="0" rIns="0" bIns="0" anchor="ctr" anchorCtr="1"/>
-            <a:lstStyle/>
-            <a:p>
-              <a:pPr algn="ctr" rtl="0">
-                <a:defRPr sz="1400"/>
-              </a:pPr>
-              <a:r>
-                <a:rPr lang="en-US" sz="1400" b="0" i="0" u="none" strike="noStrike" baseline="0">
-                  <a:solidFill>
-                    <a:sysClr val="windowText" lastClr="000000">
-                      <a:lumMod val="65000"/>
-                      <a:lumOff val="35000"/>
-                    </a:sysClr>
-                  </a:solidFill>
-                  <a:latin typeface="Aptos Narrow" panose="02110004020202020204"/>
-                </a:rPr>
-                <a:t>Number of varieties</a:t>
-              </a:r>
-            </a:p>
-          </cx:txPr>
-        </cx:title>
-        <cx:majorGridlines/>
-        <cx:tickLabels/>
-        <cx:txPr>
-          <a:bodyPr spcFirstLastPara="1" vertOverflow="ellipsis" horzOverflow="overflow" wrap="square" lIns="0" tIns="0" rIns="0" bIns="0" anchor="ctr" anchorCtr="1"/>
-          <a:lstStyle/>
-          <a:p>
-            <a:pPr algn="ctr" rtl="0">
-              <a:defRPr sz="1100"/>
-            </a:pPr>
-            <a:endParaRPr lang="en-US" sz="1100" b="0" i="0" u="none" strike="noStrike" baseline="0">
-              <a:solidFill>
-                <a:sysClr val="windowText" lastClr="000000">
-                  <a:lumMod val="65000"/>
-                  <a:lumOff val="35000"/>
-                </a:sysClr>
-              </a:solidFill>
-              <a:latin typeface="Aptos Narrow" panose="02110004020202020204"/>
-            </a:endParaRPr>
-          </a:p>
-        </cx:txPr>
-      </cx:axis>
-    </cx:plotArea>
-  </cx:chart>
-</cx:chartSpace>
-</file>
-
 <file path=xl/charts/colors1.xml><?xml version="1.0" encoding="utf-8"?>
 <cs:colorStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" meth="cycle" id="10">
   <a:schemeClr val="accent1"/>
@@ -1745,46 +1589,6 @@
 </cs:colorStyle>
 </file>
 
-<file path=xl/charts/colors4.xml><?xml version="1.0" encoding="utf-8"?>
-<cs:colorStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" meth="cycle" id="10">
-  <a:schemeClr val="accent1"/>
-  <a:schemeClr val="accent2"/>
-  <a:schemeClr val="accent3"/>
-  <a:schemeClr val="accent4"/>
-  <a:schemeClr val="accent5"/>
-  <a:schemeClr val="accent6"/>
-  <cs:variation/>
-  <cs:variation>
-    <a:lumMod val="60000"/>
-  </cs:variation>
-  <cs:variation>
-    <a:lumMod val="80000"/>
-    <a:lumOff val="20000"/>
-  </cs:variation>
-  <cs:variation>
-    <a:lumMod val="80000"/>
-  </cs:variation>
-  <cs:variation>
-    <a:lumMod val="60000"/>
-    <a:lumOff val="40000"/>
-  </cs:variation>
-  <cs:variation>
-    <a:lumMod val="50000"/>
-  </cs:variation>
-  <cs:variation>
-    <a:lumMod val="70000"/>
-    <a:lumOff val="30000"/>
-  </cs:variation>
-  <cs:variation>
-    <a:lumMod val="70000"/>
-  </cs:variation>
-  <cs:variation>
-    <a:lumMod val="50000"/>
-    <a:lumOff val="50000"/>
-  </cs:variation>
-</cs:colorStyle>
-</file>
-
 <file path=xl/charts/style1.xml><?xml version="1.0" encoding="utf-8"?>
 <cs:chartStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" id="366">
   <cs:axisTitle>
@@ -2802,514 +2606,6 @@
 </file>
 
 <file path=xl/charts/style3.xml><?xml version="1.0" encoding="utf-8"?>
-<cs:chartStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" id="366">
-  <cs:axisTitle>
-    <cs:lnRef idx="0"/>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="tx1">
-        <a:lumMod val="65000"/>
-        <a:lumOff val="35000"/>
-      </a:schemeClr>
-    </cs:fontRef>
-    <cs:defRPr sz="900"/>
-  </cs:axisTitle>
-  <cs:categoryAxis>
-    <cs:lnRef idx="0"/>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="tx1">
-        <a:lumMod val="65000"/>
-        <a:lumOff val="35000"/>
-      </a:schemeClr>
-    </cs:fontRef>
-    <cs:spPr>
-      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
-        <a:solidFill>
-          <a:schemeClr val="tx1">
-            <a:lumMod val="15000"/>
-            <a:lumOff val="85000"/>
-          </a:schemeClr>
-        </a:solidFill>
-        <a:round/>
-      </a:ln>
-    </cs:spPr>
-    <cs:defRPr sz="900"/>
-  </cs:categoryAxis>
-  <cs:chartArea mods="allowNoFillOverride allowNoLineOverride">
-    <cs:lnRef idx="0"/>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="tx1"/>
-    </cs:fontRef>
-    <cs:spPr>
-      <a:solidFill>
-        <a:schemeClr val="bg1"/>
-      </a:solidFill>
-      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
-        <a:solidFill>
-          <a:schemeClr val="tx1">
-            <a:lumMod val="15000"/>
-            <a:lumOff val="85000"/>
-          </a:schemeClr>
-        </a:solidFill>
-        <a:round/>
-      </a:ln>
-    </cs:spPr>
-    <cs:defRPr sz="1000"/>
-  </cs:chartArea>
-  <cs:dataLabel>
-    <cs:lnRef idx="0"/>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="tx1">
-        <a:lumMod val="65000"/>
-        <a:lumOff val="35000"/>
-      </a:schemeClr>
-    </cs:fontRef>
-    <cs:defRPr sz="900"/>
-  </cs:dataLabel>
-  <cs:dataLabelCallout>
-    <cs:lnRef idx="0"/>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="dk1">
-        <a:lumMod val="65000"/>
-        <a:lumOff val="35000"/>
-      </a:schemeClr>
-    </cs:fontRef>
-    <cs:spPr>
-      <a:solidFill>
-        <a:schemeClr val="lt1"/>
-      </a:solidFill>
-      <a:ln>
-        <a:solidFill>
-          <a:schemeClr val="dk1">
-            <a:lumMod val="25000"/>
-            <a:lumOff val="75000"/>
-          </a:schemeClr>
-        </a:solidFill>
-      </a:ln>
-    </cs:spPr>
-    <cs:defRPr sz="900"/>
-    <cs:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="clip" horzOverflow="clip" vert="horz" wrap="square" lIns="36576" tIns="18288" rIns="36576" bIns="18288" anchor="ctr" anchorCtr="1">
-      <a:spAutoFit/>
-    </cs:bodyPr>
-  </cs:dataLabelCallout>
-  <cs:dataPoint>
-    <cs:lnRef idx="0"/>
-    <cs:fillRef idx="0">
-      <cs:styleClr val="auto"/>
-    </cs:fillRef>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="tx1"/>
-    </cs:fontRef>
-    <cs:spPr>
-      <a:solidFill>
-        <a:schemeClr val="phClr"/>
-      </a:solidFill>
-    </cs:spPr>
-  </cs:dataPoint>
-  <cs:dataPoint3D>
-    <cs:lnRef idx="0"/>
-    <cs:fillRef idx="0">
-      <cs:styleClr val="auto"/>
-    </cs:fillRef>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="tx1"/>
-    </cs:fontRef>
-    <cs:spPr>
-      <a:solidFill>
-        <a:schemeClr val="phClr"/>
-      </a:solidFill>
-    </cs:spPr>
-  </cs:dataPoint3D>
-  <cs:dataPointLine>
-    <cs:lnRef idx="0">
-      <cs:styleClr val="auto"/>
-    </cs:lnRef>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="tx1"/>
-    </cs:fontRef>
-    <cs:spPr>
-      <a:ln w="28575" cap="rnd">
-        <a:solidFill>
-          <a:schemeClr val="phClr"/>
-        </a:solidFill>
-        <a:round/>
-      </a:ln>
-    </cs:spPr>
-  </cs:dataPointLine>
-  <cs:dataPointMarker>
-    <cs:lnRef idx="0"/>
-    <cs:fillRef idx="0">
-      <cs:styleClr val="auto"/>
-    </cs:fillRef>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="tx1"/>
-    </cs:fontRef>
-    <cs:spPr>
-      <a:solidFill>
-        <a:schemeClr val="phClr"/>
-      </a:solidFill>
-      <a:ln w="9525">
-        <a:solidFill>
-          <a:schemeClr val="lt1"/>
-        </a:solidFill>
-      </a:ln>
-    </cs:spPr>
-  </cs:dataPointMarker>
-  <cs:dataPointMarkerLayout symbol="circle" size="5"/>
-  <cs:dataPointWireframe>
-    <cs:lnRef idx="0">
-      <cs:styleClr val="auto"/>
-    </cs:lnRef>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="tx1"/>
-    </cs:fontRef>
-    <cs:spPr>
-      <a:ln w="28575" cap="rnd">
-        <a:solidFill>
-          <a:schemeClr val="phClr"/>
-        </a:solidFill>
-        <a:round/>
-      </a:ln>
-    </cs:spPr>
-  </cs:dataPointWireframe>
-  <cs:dataTable>
-    <cs:lnRef idx="0"/>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="tx1">
-        <a:lumMod val="65000"/>
-        <a:lumOff val="35000"/>
-      </a:schemeClr>
-    </cs:fontRef>
-    <cs:spPr>
-      <a:ln w="9525">
-        <a:solidFill>
-          <a:schemeClr val="tx1">
-            <a:lumMod val="15000"/>
-            <a:lumOff val="85000"/>
-          </a:schemeClr>
-        </a:solidFill>
-      </a:ln>
-    </cs:spPr>
-    <cs:defRPr sz="900"/>
-  </cs:dataTable>
-  <cs:downBar>
-    <cs:lnRef idx="0"/>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="dk1"/>
-    </cs:fontRef>
-    <cs:spPr>
-      <a:solidFill>
-        <a:schemeClr val="dk1">
-          <a:lumMod val="65000"/>
-          <a:lumOff val="35000"/>
-        </a:schemeClr>
-      </a:solidFill>
-      <a:ln w="9525">
-        <a:solidFill>
-          <a:schemeClr val="tx1">
-            <a:lumMod val="65000"/>
-            <a:lumOff val="35000"/>
-          </a:schemeClr>
-        </a:solidFill>
-      </a:ln>
-    </cs:spPr>
-  </cs:downBar>
-  <cs:dropLine>
-    <cs:lnRef idx="0"/>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="tx1"/>
-    </cs:fontRef>
-    <cs:spPr>
-      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
-        <a:solidFill>
-          <a:schemeClr val="tx1">
-            <a:lumMod val="35000"/>
-            <a:lumOff val="65000"/>
-          </a:schemeClr>
-        </a:solidFill>
-        <a:round/>
-      </a:ln>
-    </cs:spPr>
-  </cs:dropLine>
-  <cs:errorBar>
-    <cs:lnRef idx="0"/>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="tx1"/>
-    </cs:fontRef>
-    <cs:spPr>
-      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
-        <a:solidFill>
-          <a:schemeClr val="tx1">
-            <a:lumMod val="65000"/>
-            <a:lumOff val="35000"/>
-          </a:schemeClr>
-        </a:solidFill>
-        <a:round/>
-      </a:ln>
-    </cs:spPr>
-  </cs:errorBar>
-  <cs:floor>
-    <cs:lnRef idx="0"/>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="tx1"/>
-    </cs:fontRef>
-  </cs:floor>
-  <cs:gridlineMajor>
-    <cs:lnRef idx="0"/>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="tx1"/>
-    </cs:fontRef>
-    <cs:spPr>
-      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
-        <a:solidFill>
-          <a:schemeClr val="tx1">
-            <a:lumMod val="15000"/>
-            <a:lumOff val="85000"/>
-          </a:schemeClr>
-        </a:solidFill>
-        <a:round/>
-      </a:ln>
-    </cs:spPr>
-  </cs:gridlineMajor>
-  <cs:gridlineMinor>
-    <cs:lnRef idx="0"/>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="tx1"/>
-    </cs:fontRef>
-    <cs:spPr>
-      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
-        <a:solidFill>
-          <a:schemeClr val="tx1">
-            <a:lumMod val="15000"/>
-            <a:lumOff val="85000"/>
-          </a:schemeClr>
-        </a:solidFill>
-        <a:round/>
-      </a:ln>
-    </cs:spPr>
-  </cs:gridlineMinor>
-  <cs:hiLoLine>
-    <cs:lnRef idx="0"/>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="tx1"/>
-    </cs:fontRef>
-    <cs:spPr>
-      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
-        <a:solidFill>
-          <a:schemeClr val="tx1">
-            <a:lumMod val="75000"/>
-            <a:lumOff val="25000"/>
-          </a:schemeClr>
-        </a:solidFill>
-        <a:round/>
-      </a:ln>
-    </cs:spPr>
-  </cs:hiLoLine>
-  <cs:leaderLine>
-    <cs:lnRef idx="0"/>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="tx1"/>
-    </cs:fontRef>
-    <cs:spPr>
-      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
-        <a:solidFill>
-          <a:schemeClr val="tx1">
-            <a:lumMod val="35000"/>
-            <a:lumOff val="65000"/>
-          </a:schemeClr>
-        </a:solidFill>
-        <a:round/>
-      </a:ln>
-    </cs:spPr>
-  </cs:leaderLine>
-  <cs:legend>
-    <cs:lnRef idx="0"/>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="tx1">
-        <a:lumMod val="65000"/>
-        <a:lumOff val="35000"/>
-      </a:schemeClr>
-    </cs:fontRef>
-    <cs:defRPr sz="900"/>
-  </cs:legend>
-  <cs:plotArea mods="allowNoFillOverride allowNoLineOverride">
-    <cs:lnRef idx="0"/>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="tx1"/>
-    </cs:fontRef>
-  </cs:plotArea>
-  <cs:plotArea3D mods="allowNoFillOverride allowNoLineOverride">
-    <cs:lnRef idx="0"/>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="tx1"/>
-    </cs:fontRef>
-  </cs:plotArea3D>
-  <cs:seriesAxis>
-    <cs:lnRef idx="0"/>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="tx1">
-        <a:lumMod val="65000"/>
-        <a:lumOff val="35000"/>
-      </a:schemeClr>
-    </cs:fontRef>
-    <cs:spPr>
-      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
-        <a:solidFill>
-          <a:schemeClr val="tx1">
-            <a:lumMod val="15000"/>
-            <a:lumOff val="85000"/>
-          </a:schemeClr>
-        </a:solidFill>
-        <a:round/>
-      </a:ln>
-    </cs:spPr>
-    <cs:defRPr sz="900"/>
-  </cs:seriesAxis>
-  <cs:seriesLine>
-    <cs:lnRef idx="0"/>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="tx1"/>
-    </cs:fontRef>
-    <cs:spPr>
-      <a:ln w="9525" cap="flat">
-        <a:solidFill>
-          <a:srgbClr val="D9D9D9"/>
-        </a:solidFill>
-        <a:round/>
-      </a:ln>
-    </cs:spPr>
-  </cs:seriesLine>
-  <cs:title>
-    <cs:lnRef idx="0"/>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="tx1">
-        <a:lumMod val="65000"/>
-        <a:lumOff val="35000"/>
-      </a:schemeClr>
-    </cs:fontRef>
-    <cs:defRPr sz="1400"/>
-  </cs:title>
-  <cs:trendline>
-    <cs:lnRef idx="0">
-      <cs:styleClr val="auto"/>
-    </cs:lnRef>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="tx1"/>
-    </cs:fontRef>
-    <cs:spPr>
-      <a:ln w="19050" cap="rnd">
-        <a:solidFill>
-          <a:schemeClr val="phClr"/>
-        </a:solidFill>
-        <a:prstDash val="sysDash"/>
-      </a:ln>
-    </cs:spPr>
-  </cs:trendline>
-  <cs:trendlineLabel>
-    <cs:lnRef idx="0"/>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="tx1">
-        <a:lumMod val="65000"/>
-        <a:lumOff val="35000"/>
-      </a:schemeClr>
-    </cs:fontRef>
-    <cs:defRPr sz="900"/>
-  </cs:trendlineLabel>
-  <cs:upBar>
-    <cs:lnRef idx="0"/>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="dk1"/>
-    </cs:fontRef>
-    <cs:spPr>
-      <a:solidFill>
-        <a:schemeClr val="lt1"/>
-      </a:solidFill>
-      <a:ln w="9525">
-        <a:solidFill>
-          <a:schemeClr val="tx1">
-            <a:lumMod val="15000"/>
-            <a:lumOff val="85000"/>
-          </a:schemeClr>
-        </a:solidFill>
-      </a:ln>
-    </cs:spPr>
-  </cs:upBar>
-  <cs:valueAxis>
-    <cs:lnRef idx="0"/>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="tx1">
-        <a:lumMod val="65000"/>
-        <a:lumOff val="35000"/>
-      </a:schemeClr>
-    </cs:fontRef>
-    <cs:defRPr sz="900"/>
-  </cs:valueAxis>
-  <cs:wall>
-    <cs:lnRef idx="0"/>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="tx1"/>
-    </cs:fontRef>
-  </cs:wall>
-</cs:chartStyle>
-</file>
-
-<file path=xl/charts/style4.xml><?xml version="1.0" encoding="utf-8"?>
 <cs:chartStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" id="366">
   <cs:axisTitle>
     <cs:lnRef idx="0"/>
@@ -4024,89 +3320,6 @@
             <a:xfrm>
               <a:off x="927100" y="5803900"/>
               <a:ext cx="5156200" cy="2794000"/>
-            </a:xfrm>
-            <a:prstGeom prst="rect">
-              <a:avLst/>
-            </a:prstGeom>
-            <a:solidFill>
-              <a:prstClr val="white"/>
-            </a:solidFill>
-            <a:ln w="1">
-              <a:solidFill>
-                <a:prstClr val="green"/>
-              </a:solidFill>
-            </a:ln>
-          </xdr:spPr>
-          <xdr:txBody>
-            <a:bodyPr vertOverflow="clip" horzOverflow="clip"/>
-            <a:lstStyle/>
-            <a:p>
-              <a:r>
-                <a:rPr lang="en-US" sz="1100"/>
-                <a:t>This chart isn't available in your version of Excel.
-Editing this shape or saving this workbook into a different file format will permanently break the chart.</a:t>
-              </a:r>
-            </a:p>
-          </xdr:txBody>
-        </xdr:sp>
-      </mc:Fallback>
-    </mc:AlternateContent>
-    <xdr:clientData/>
-  </xdr:twoCellAnchor>
-</xdr:wsDr>
-</file>
-
-<file path=xl/drawings/drawing2.xml><?xml version="1.0" encoding="utf-8"?>
-<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-  <xdr:twoCellAnchor>
-    <xdr:from>
-      <xdr:col>3</xdr:col>
-      <xdr:colOff>57150</xdr:colOff>
-      <xdr:row>3</xdr:row>
-      <xdr:rowOff>133350</xdr:rowOff>
-    </xdr:from>
-    <xdr:to>
-      <xdr:col>12</xdr:col>
-      <xdr:colOff>584200</xdr:colOff>
-      <xdr:row>23</xdr:row>
-      <xdr:rowOff>114300</xdr:rowOff>
-    </xdr:to>
-    <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-      <mc:Choice xmlns:cx1="http://schemas.microsoft.com/office/drawing/2015/9/8/chartex" Requires="cx1">
-        <xdr:graphicFrame macro="">
-          <xdr:nvGraphicFramePr>
-            <xdr:cNvPr id="5" name="Chart 4">
-              <a:extLst>
-                <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-                  <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{84D90639-4167-A7B6-A9A2-B61A3671B4FA}"/>
-                </a:ext>
-              </a:extLst>
-            </xdr:cNvPr>
-            <xdr:cNvGraphicFramePr/>
-          </xdr:nvGraphicFramePr>
-          <xdr:xfrm>
-            <a:off x="0" y="0"/>
-            <a:ext cx="0" cy="0"/>
-          </xdr:xfrm>
-          <a:graphic>
-            <a:graphicData uri="http://schemas.microsoft.com/office/drawing/2014/chartex">
-              <cx:chart xmlns:cx="http://schemas.microsoft.com/office/drawing/2014/chartex" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
-            </a:graphicData>
-          </a:graphic>
-        </xdr:graphicFrame>
-      </mc:Choice>
-      <mc:Fallback>
-        <xdr:sp macro="" textlink="">
-          <xdr:nvSpPr>
-            <xdr:cNvPr id="0" name=""/>
-            <xdr:cNvSpPr>
-              <a:spLocks noTextEdit="1"/>
-            </xdr:cNvSpPr>
-          </xdr:nvSpPr>
-          <xdr:spPr>
-            <a:xfrm>
-              <a:off x="2533650" y="755650"/>
-              <a:ext cx="7956550" cy="4044950"/>
             </a:xfrm>
             <a:prstGeom prst="rect">
               <a:avLst/>
@@ -4722,7 +3935,6 @@
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <drawing r:id="rId1"/>
 </worksheet>
 </file>
 

</xml_diff>

<commit_message>
Embed SharePoint answer workbooks for bank Questions 1-2
Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01TNVxQFJXojPDm4Z5hNnmdq
</commit_message>
<xml_diff>
--- a/textbook_examples/mod01_descriptives.xlsx
+++ b/textbook_examples/mod01_descriptives.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://usaskca1-my.sharepoint.com/personal/pjs998_usask_ca/Documents/Teaching/261/2026/textbook_261/textbook_examples/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="159" documentId="8_{40A48D82-9896-1D40-A33B-1B9FE8A350F6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{FB1EDDDA-D220-7F48-80FF-7FEA6C4C0826}"/>
+  <xr:revisionPtr revIDLastSave="160" documentId="8_{40A48D82-9896-1D40-A33B-1B9FE8A350F6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{CF648DDB-989D-C348-971D-BBC5C44E2E61}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="38400" windowHeight="21600" activeTab="9" xr2:uid="{E0A39ED0-7C98-1C4C-834F-3D01DA12686E}"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="38400" windowHeight="21600" activeTab="3" xr2:uid="{E0A39ED0-7C98-1C4C-834F-3D01DA12686E}"/>
   </bookViews>
   <sheets>
     <sheet name="README" sheetId="3" r:id="rId1"/>
@@ -4354,7 +4354,7 @@
         <v>34006434.399999999</v>
       </c>
       <c r="F2" s="23" t="s">
-        <v>44</v>
+        <v>63</v>
       </c>
       <c r="G2" s="23"/>
     </row>

</xml_diff>